<commit_message>
P&ID revision: classes A3/S3/F1, SIF-109 redefinition, P-119, steam/thermal reliefs, slop wax hot route
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013qGZUcwwWBAcAEPeh7Toud
</commit_message>
<xml_diff>
--- a/deliverables/03-layout-piping/CFU-000-PI-SPC-001_Piping-Class-Summary.xlsx
+++ b/deliverables/03-layout-piping/CFU-000-PI-SPC-001_Piping-Class-Summary.xlsx
@@ -12,9 +12,9 @@
     <sheet name="Rating Exceptions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Classes'!$A$4:$P$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'P-T Ratings'!$A$4:$R$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Rating Exceptions'!$A$4:$A$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Classes'!$A$4:$P$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'P-T Ratings'!$A$4:$R$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Rating Exceptions'!$A$4:$A$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -630,13 +630,13 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="O5" t="n">
         <v>14.5</v>
       </c>
       <c r="P5" t="n">
-        <v>290</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6">
@@ -774,7 +774,7 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="O7" t="n">
         <v>41</v>
@@ -846,7 +846,7 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="O8" t="n">
         <v>41</v>
@@ -1002,17 +1002,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>A3</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>150#</t>
+          <t>300#</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Carbon steel ASTM A106 Gr.B</t>
+          <t>Carbon steel, HIC-resistant (NACE MR0103), PWHT</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1021,75 +1021,75 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>1.5</v>
+        <v>6</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>LP / MP steam, condensate</t>
+          <t>Wash water / brine / sour water above 150# rating (desalter pressure)</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>A105 RF</t>
+          <t>A105N RF, HB &lt;= 200</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Gate/globe A216 WCB, trim 8</t>
+          <t>Gate/globe A216 WCB NACE, trim 316/stellite</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>SPW 304/graphite</t>
+          <t>SPW 316L/graphite, inner + outer ring</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>A193 B7 / A194 2H</t>
+          <t>A193 B7M / A194 2HM</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Weldolet / tee</t>
+          <t>Weldolet / reinforced tee, PWHT</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Sch 40 / STD</t>
+          <t>Sch 80 &lt;= 2", Sch 40 / XS &gt;= 3"</t>
         </is>
       </c>
       <c r="N11" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="O11" t="n">
-        <v>13</v>
+        <v>24.5</v>
       </c>
       <c r="P11" t="n">
-        <v>380</v>
+        <v>165</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>600#</t>
+          <t>150#</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.25Cr-1/2Mo ASTM A335 P11</t>
+          <t>Carbon steel ASTM A106 Gr.B</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -1097,20 +1097,20 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>HP steam 41 barg / 400 C</t>
+          <t>LP / MP steam, condensate</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>450</v>
+        <v>400</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>A182 F11 Cl.2 RF</t>
+          <t>A105 RF</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Gate/globe A217 WC6, trim 8</t>
+          <t>Gate/globe A216 WCB, trim 8</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1125,43 +1125,43 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Weldolet, PWHT</t>
+          <t>Weldolet / tee</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Sch 80</t>
+          <t>Sch 40 / STD</t>
         </is>
       </c>
       <c r="N12" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="O12" t="n">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="P12" t="n">
-        <v>430</v>
+        <v>380</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>150#</t>
+          <t>600#</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Carbon steel (cement-lined for CW &gt;= 12")</t>
+          <t>1.25Cr-1/2Mo ASTM A335 P11</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -1169,25 +1169,25 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Cooling water, utility water, LP BFW</t>
+          <t>HP steam 41 barg / 400 C</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>120</v>
+        <v>450</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>A105 RF</t>
+          <t>A182 F11 Cl.2 RF</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Butterfly (&gt;= 6"), gate (&lt;= 4")</t>
+          <t>Gate/globe A217 WC6, trim 8</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Non-asbestos fibre</t>
+          <t>SPW 304/graphite</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1197,100 +1197,100 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Tee / weldolet</t>
+          <t>Weldolet, PWHT</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>STD</t>
+          <t>Sch 80</t>
         </is>
       </c>
       <c r="N13" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="O13" t="n">
-        <v>8.199999999999999</v>
+        <v>46</v>
       </c>
       <c r="P13" t="n">
-        <v>75</v>
+        <v>430</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>S3</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>150#</t>
+          <t>300#</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>SS304 (IA) / galvanised CS (N2)</t>
+          <t>Carbon steel ASTM A106 Gr.B</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Instrument air, nitrogen</t>
+          <t>MP steam 10.3 barg / 250-290 C design (exceeds S1)</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>A182 F304 RF / screwed &lt;= 1-1/2"</t>
+          <t>A105 RF</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Ball SS316</t>
+          <t>Gate/globe A216 WCB, trim 8 (stellite seats)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>PTFE / SPW 304</t>
+          <t>SPW 304/graphite, inner ring</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>A193 B8 / A194 8</t>
+          <t>A193 B7 / A194 2H</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Tee</t>
+          <t>Weldolet / tee</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Sch 10S / 40S</t>
+          <t>Sch 40 / STD, Sch 80 &lt;= 1-1/2"</t>
         </is>
       </c>
       <c r="N14" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="O14" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="P14" t="n">
-        <v>65</v>
+        <v>290</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>V1</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1300,12 +1300,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5Cr-1/2Mo ASTM A335 P5</t>
+          <t>Carbon steel, killed, impact-tested (A333 Gr.6)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -1313,54 +1313,270 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Vacuum vapour lines (C-201 OH); transfer line &gt; 400 C -&gt; B3</t>
+          <t>Flare / relief headers, -29 to 350 C</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>400</v>
+        <v>350</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>A182 F5 RF</t>
+          <t>A350 LF2 RF</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Gate A217 C5 (vacuum service, bellows/stem purge)</t>
+          <t>Gate A352 LCC (CSO/CSC per relief philosophy)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>SPW 321/graphite</t>
+          <t>SPW 304/graphite, inner ring</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>A193 B7 / A194 4</t>
+          <t>A320 L7 / A194 4</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Reinforced, full vacuum design</t>
+          <t>Lateral 45 deg into header top; reinforced</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>STD / per vacuum collapse</t>
+          <t>STD, min. Sch 40 (acoustic fatigue check for large laterals)</t>
         </is>
       </c>
       <c r="N15" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="O15" t="n">
         <v>3.5</v>
       </c>
       <c r="P15" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>U1</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>150#</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Carbon steel (cement-lined for CW &gt;= 12")</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Cooling water, utility water, LP BFW</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>120</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>A105 RF</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Butterfly (&gt;= 6"), gate (&lt;= 4")</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Non-asbestos fibre</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>A193 B7 / A194 2H</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Tee / weldolet</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>STD</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>10</v>
+      </c>
+      <c r="O16" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="P16" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>U2</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>150#</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>SS304 (IA) / galvanised CS (N2)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Instrument air, nitrogen</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>100</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>A182 F304 RF / screwed &lt;= 1-1/2"</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Ball SS316</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>PTFE / SPW 304</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>A193 B8 / A194 8</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Tee</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Sch 10S / 40S</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>2</v>
+      </c>
+      <c r="O17" t="n">
+        <v>10</v>
+      </c>
+      <c r="P17" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>150#</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>5Cr-1/2Mo ASTM A335 P5</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Vacuum vapour lines (C-201 OH); transfer line &gt; 400 C -&gt; B3</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>400</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>A182 F5 RF</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Gate A217 C5 (vacuum service, bellows/stem purge)</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>SPW 321/graphite</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>A193 B7 / A194 4</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Reinforced, full vacuum design</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>STD / per vacuum collapse</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>1</v>
+      </c>
+      <c r="O18" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="P18" t="n">
         <v>180</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:P15"/>
+  <autoFilter ref="A4:P18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1371,7 +1587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R15"/>
+  <dimension ref="A1:R18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1875,12 +2091,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>A3</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>150#</t>
+          <t>300#</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1889,241 +2105,241 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>19.6</v>
+        <v>51.1</v>
       </c>
       <c r="E11" t="n">
-        <v>19.2</v>
+        <v>50.1</v>
       </c>
       <c r="F11" t="n">
-        <v>17.7</v>
+        <v>46.6</v>
       </c>
       <c r="G11" t="n">
-        <v>15.8</v>
+        <v>45.1</v>
       </c>
       <c r="H11" t="n">
-        <v>13.8</v>
+        <v>43.8</v>
       </c>
       <c r="I11" t="n">
-        <v>12.1</v>
+        <v>41.9</v>
       </c>
       <c r="J11" t="n">
-        <v>10.2</v>
+        <v>39.8</v>
       </c>
       <c r="K11" t="n">
-        <v>9.300000000000001</v>
+        <v>38.7</v>
       </c>
       <c r="L11" t="n">
-        <v>8.4</v>
+        <v>37.6</v>
       </c>
       <c r="M11" t="n">
-        <v>7.4</v>
+        <v>36.4</v>
       </c>
       <c r="N11" t="n">
-        <v>6.5</v>
+        <v>34.7</v>
       </c>
       <c r="O11" t="n">
-        <v>5.5</v>
+        <v>28.8</v>
       </c>
       <c r="P11" t="n">
-        <v>4.6</v>
+        <v>23</v>
       </c>
       <c r="Q11" t="n">
-        <v>3.7</v>
+        <v>17.4</v>
       </c>
       <c r="R11" t="n">
-        <v>2.8</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>600#</t>
+          <t>150#</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>103.4</v>
+        <v>19.6</v>
       </c>
       <c r="E12" t="n">
-        <v>103.4</v>
+        <v>19.2</v>
       </c>
       <c r="F12" t="n">
-        <v>103</v>
+        <v>17.7</v>
       </c>
       <c r="G12" t="n">
-        <v>99.5</v>
+        <v>15.8</v>
       </c>
       <c r="H12" t="n">
-        <v>97.2</v>
+        <v>13.8</v>
       </c>
       <c r="I12" t="n">
-        <v>92.7</v>
+        <v>12.1</v>
       </c>
       <c r="J12" t="n">
-        <v>85.7</v>
+        <v>10.2</v>
       </c>
       <c r="K12" t="n">
-        <v>82.59999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="L12" t="n">
-        <v>80.40000000000001</v>
+        <v>8.4</v>
       </c>
       <c r="M12" t="n">
-        <v>77.59999999999999</v>
+        <v>7.4</v>
       </c>
       <c r="N12" t="n">
-        <v>72.90000000000001</v>
+        <v>6.5</v>
       </c>
       <c r="O12" t="n">
-        <v>70</v>
+        <v>5.5</v>
       </c>
       <c r="P12" t="n">
-        <v>67.7</v>
+        <v>4.6</v>
       </c>
       <c r="Q12" t="n">
-        <v>63.4</v>
+        <v>3.7</v>
       </c>
       <c r="R12" t="n">
-        <v>46.8</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>150#</t>
+          <t>600#</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>19.6</v>
+        <v>103.4</v>
       </c>
       <c r="E13" t="n">
-        <v>19.2</v>
+        <v>103.4</v>
       </c>
       <c r="F13" t="n">
-        <v>17.7</v>
+        <v>103</v>
       </c>
       <c r="G13" t="n">
-        <v>15.8</v>
+        <v>99.5</v>
       </c>
       <c r="H13" t="n">
-        <v>13.8</v>
+        <v>97.2</v>
       </c>
       <c r="I13" t="n">
-        <v>12.1</v>
+        <v>92.7</v>
       </c>
       <c r="J13" t="n">
-        <v>10.2</v>
+        <v>85.7</v>
       </c>
       <c r="K13" t="n">
-        <v>9.300000000000001</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="L13" t="n">
-        <v>8.4</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="M13" t="n">
-        <v>7.4</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="N13" t="n">
-        <v>6.5</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="O13" t="n">
-        <v>5.5</v>
+        <v>70</v>
       </c>
       <c r="P13" t="n">
-        <v>4.6</v>
+        <v>67.7</v>
       </c>
       <c r="Q13" t="n">
-        <v>3.7</v>
+        <v>63.4</v>
       </c>
       <c r="R13" t="n">
-        <v>2.8</v>
+        <v>46.8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>S3</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>150#</t>
+          <t>300#</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>19</v>
+        <v>51.1</v>
       </c>
       <c r="E14" t="n">
-        <v>18.3</v>
+        <v>50.1</v>
       </c>
       <c r="F14" t="n">
-        <v>15.7</v>
+        <v>46.6</v>
       </c>
       <c r="G14" t="n">
-        <v>14.2</v>
+        <v>45.1</v>
       </c>
       <c r="H14" t="n">
-        <v>13.2</v>
+        <v>43.8</v>
       </c>
       <c r="I14" t="n">
-        <v>12.1</v>
+        <v>41.9</v>
       </c>
       <c r="J14" t="n">
-        <v>10.2</v>
+        <v>39.8</v>
       </c>
       <c r="K14" t="n">
-        <v>9.300000000000001</v>
+        <v>38.7</v>
       </c>
       <c r="L14" t="n">
-        <v>8.4</v>
+        <v>37.6</v>
       </c>
       <c r="M14" t="n">
-        <v>7.4</v>
+        <v>36.4</v>
       </c>
       <c r="N14" t="n">
-        <v>6.5</v>
+        <v>34.7</v>
       </c>
       <c r="O14" t="n">
-        <v>5.5</v>
+        <v>28.8</v>
       </c>
       <c r="P14" t="n">
-        <v>4.6</v>
+        <v>23</v>
       </c>
       <c r="Q14" t="n">
-        <v>3.7</v>
+        <v>17.4</v>
       </c>
       <c r="R14" t="n">
-        <v>2.8</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>V1</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2133,14 +2349,14 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>20</v>
+        <v>19.6</v>
       </c>
       <c r="E15" t="n">
-        <v>19.5</v>
+        <v>19.2</v>
       </c>
       <c r="F15" t="n">
         <v>17.7</v>
@@ -2182,8 +2398,194 @@
         <v>2.8</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>U1</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>150#</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="E16" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="F16" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="G16" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="H16" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="I16" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="J16" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="K16" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="L16" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="M16" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="N16" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O16" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="P16" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="R16" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>U2</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>150#</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>19</v>
+      </c>
+      <c r="E17" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="F17" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="G17" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="H17" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="I17" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="J17" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="K17" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="L17" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="M17" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="N17" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O17" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="P17" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="R17" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>150#</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>20</v>
+      </c>
+      <c r="E18" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="F18" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="G18" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="H18" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="I18" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="J18" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="K18" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="L18" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="M18" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="N18" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O18" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="P18" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="R18" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:R15"/>
+  <autoFilter ref="A4:R18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2194,7 +2596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -2221,78 +2623,9 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>6"-MS-100-056-S1-H: design 13.0 barg @ 290.0 C exceeds class S1 rating 10.6 barg</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>1"-BD-100-057-S1-N: design 13.0 barg @ 290.0 C exceeds class S1 rating 10.6 barg</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>8"-MS-100-151-S1-H: design 13.0 barg @ 280 C exceeds class S1 rating 11.0 barg</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>3"-MS-200-018-S1-H: design 12.0 barg @ 280 C exceeds class S1 rating 11.0 barg</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>4"-MS-200-032-S1-H: design 12.0 barg @ 280 C exceeds class S1 rating 11.0 barg</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>6"-MS-200-046-S1-H: design 12.0 barg @ 280 C exceeds class S1 rating 11.0 barg</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>3"-MS-200-047-S1-H: design 12.0 barg @ 280 C exceeds class S1 rating 11.0 barg</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2"-MS-200-048-S1-H: design 12.0 barg @ 280 C exceeds class S1 rating 11.0 barg</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>10"-MS-900-008-S1-H: design 12.0 barg @ 280 C exceeds class S1 rating 11.0 barg</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>6"-MS-900-010-S1-H: design 12.0 barg @ 280 C exceeds class S1 rating 11.0 barg</t>
-        </is>
-      </c>
-    </row>
+    <row r="5"/>
   </sheetData>
-  <autoFilter ref="A4:A14"/>
+  <autoFilter ref="A4:A4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>